<commit_message>
Use Visual Studio 2022 and add XAMPP to the software list
Visual Studio 2022 Community replaces 2026 everywhere because the training PCs run Windows 10. XAMPP 8.5.12 is added to the landing, README, AGENTS and skill software lists. The dev-tools, is-code and MAPO plans are updated; no practice referenced the old IDE or needed a XAMPP step.
</commit_message>
<xml_diff>
--- a/courses/2/dev-tools/dist/Учебный_план_Инструментальные_средства_разработки_ПО.xlsx
+++ b/courses/2/dev-tools/dist/Учебный_план_Инструментальные_средства_разработки_ПО.xlsx
@@ -247,7 +247,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 1. Настройка VS Code; Настройка Visual Studio 2026</t>
+          <t xml:space="preserve">Практика 1. Настройка VS Code; Настройка Visual Studio 2022</t>
         </is>
       </c>
       <c r="D8" s="6">
@@ -277,7 +277,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 3. Visual Studio 2026 Community</t>
+          <t xml:space="preserve">Лекция 3. Visual Studio 2022 Community</t>
         </is>
       </c>
       <c r="D9" s="6">

</xml_diff>